<commit_message>
xcel sheet updated with department and usn in that
</commit_message>
<xml_diff>
--- a/src/assets/studenttemplate.xlsx
+++ b/src/assets/studenttemplate.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99253161-D65A-451A-91E5-931239EF0609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ganesh\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B3D20A9-9185-41DE-8801-21C58262585A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Students" sheetId="1" r:id="rId1"/>
@@ -22,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -42,17 +45,17 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>satya</t>
+    <t>USN</t>
   </si>
   <si>
-    <t>satya@example.com</t>
+    <t>Department</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -65,6 +68,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -415,15 +419,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -433,25 +439,22 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3">
-        <v>98654321</v>
-      </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{B38BB9A6-F3E6-4483-81FB-5B47DA20ECC2}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>